<commit_message>
Added new RDF data schemes and visual schemes for environment-table19-20, and fixed XLSX spreadsheets for environment-table19-20
</commit_message>
<xml_diff>
--- a/sources/table_normalization/xlsx/environment-table19.xlsx
+++ b/sources/table_normalization/xlsx/environment-table19.xlsx
@@ -548,7 +548,7 @@
     <xf numFmtId="9" fontId="12" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="90">
+  <cellXfs count="87">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
@@ -687,25 +687,21 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="6" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -753,11 +749,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1450,33 +1443,32 @@
       <c r="A4" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="64"/>
-      <c r="C4" s="65"/>
-      <c r="D4" s="65"/>
-      <c r="E4" s="66"/>
-      <c r="F4" s="67" t="s">
+      <c r="C4" s="13"/>
+      <c r="D4" s="13"/>
+      <c r="E4" s="14"/>
+      <c r="F4" s="64" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="20.149999999999999" customHeight="1">
-      <c r="A5" s="68" t="s">
+      <c r="A5" s="65" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="84" t="s">
+      <c r="B5" s="82" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="78" t="s">
+      <c r="C5" s="76" t="s">
         <v>5</v>
       </c>
-      <c r="D5" s="79"/>
-      <c r="E5" s="80"/>
-      <c r="F5" s="88" t="s">
+      <c r="D5" s="77"/>
+      <c r="E5" s="78"/>
+      <c r="F5" s="68" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="72.75" customHeight="1">
-      <c r="A6" s="69"/>
-      <c r="B6" s="85"/>
+      <c r="A6" s="86"/>
+      <c r="B6" s="83"/>
       <c r="C6" s="19" t="s">
         <v>7</v>
       </c>
@@ -1486,10 +1478,10 @@
       <c r="E6" s="19" t="s">
         <v>9</v>
       </c>
-      <c r="F6" s="89"/>
+      <c r="F6" s="69"/>
     </row>
     <row r="7" spans="1:6" ht="15.9" customHeight="1">
-      <c r="A7" s="72" t="s">
+      <c r="A7" s="70" t="s">
         <v>10</v>
       </c>
       <c r="B7" s="21" t="s">
@@ -1510,7 +1502,7 @@
       </c>
     </row>
     <row r="8" spans="1:6" ht="15.9" customHeight="1">
-      <c r="A8" s="72"/>
+      <c r="A8" s="70"/>
       <c r="B8" s="24" t="s">
         <v>12</v>
       </c>
@@ -1529,7 +1521,7 @@
       </c>
     </row>
     <row r="9" spans="1:6" ht="15.9" customHeight="1">
-      <c r="A9" s="72"/>
+      <c r="A9" s="70"/>
       <c r="B9" s="21" t="s">
         <v>13</v>
       </c>
@@ -1548,7 +1540,7 @@
       </c>
     </row>
     <row r="10" spans="1:6" ht="15.9" customHeight="1">
-      <c r="A10" s="72"/>
+      <c r="A10" s="70"/>
       <c r="B10" s="24" t="s">
         <v>14</v>
       </c>
@@ -1567,7 +1559,7 @@
       </c>
     </row>
     <row r="11" spans="1:6" ht="15.9" customHeight="1">
-      <c r="A11" s="72"/>
+      <c r="A11" s="70"/>
       <c r="B11" s="21" t="s">
         <v>15</v>
       </c>
@@ -1586,7 +1578,7 @@
       </c>
     </row>
     <row r="12" spans="1:6" ht="15.9" customHeight="1">
-      <c r="A12" s="73"/>
+      <c r="A12" s="71"/>
       <c r="B12" s="27" t="s">
         <v>6</v>
       </c>
@@ -1608,7 +1600,7 @@
       </c>
     </row>
     <row r="13" spans="1:6" ht="15.9" customHeight="1">
-      <c r="A13" s="72" t="s">
+      <c r="A13" s="70" t="s">
         <v>16</v>
       </c>
       <c r="B13" s="21" t="s">
@@ -1629,7 +1621,7 @@
       </c>
     </row>
     <row r="14" spans="1:6" ht="15.9" customHeight="1">
-      <c r="A14" s="72"/>
+      <c r="A14" s="70"/>
       <c r="B14" s="24" t="s">
         <v>12</v>
       </c>
@@ -1648,7 +1640,7 @@
       </c>
     </row>
     <row r="15" spans="1:6" ht="15.9" customHeight="1">
-      <c r="A15" s="72"/>
+      <c r="A15" s="70"/>
       <c r="B15" s="21" t="s">
         <v>13</v>
       </c>
@@ -1667,7 +1659,7 @@
       </c>
     </row>
     <row r="16" spans="1:6" ht="15.9" customHeight="1">
-      <c r="A16" s="72"/>
+      <c r="A16" s="70"/>
       <c r="B16" s="24" t="s">
         <v>14</v>
       </c>
@@ -1686,7 +1678,7 @@
       </c>
     </row>
     <row r="17" spans="1:6" ht="15.9" customHeight="1">
-      <c r="A17" s="72"/>
+      <c r="A17" s="70"/>
       <c r="B17" s="21" t="str">
         <f>$B$11</f>
         <v>Breeding of GM or HM</v>
@@ -1706,7 +1698,7 @@
       </c>
     </row>
     <row r="18" spans="1:6" ht="15.9" customHeight="1">
-      <c r="A18" s="73"/>
+      <c r="A18" s="71"/>
       <c r="B18" s="27" t="s">
         <v>6</v>
       </c>
@@ -2208,7 +2200,7 @@
       </c>
     </row>
     <row r="43" spans="1:6" ht="15.9" customHeight="1">
-      <c r="A43" s="72" t="s">
+      <c r="A43" s="70" t="s">
         <v>22</v>
       </c>
       <c r="B43" s="21" t="s">
@@ -2229,7 +2221,7 @@
       </c>
     </row>
     <row r="44" spans="1:6" ht="15.9" customHeight="1">
-      <c r="A44" s="72"/>
+      <c r="A44" s="70"/>
       <c r="B44" s="24" t="s">
         <v>12</v>
       </c>
@@ -2248,7 +2240,7 @@
       </c>
     </row>
     <row r="45" spans="1:6" ht="15.9" customHeight="1">
-      <c r="A45" s="72"/>
+      <c r="A45" s="70"/>
       <c r="B45" s="21" t="s">
         <v>13</v>
       </c>
@@ -2267,7 +2259,7 @@
       </c>
     </row>
     <row r="46" spans="1:6" ht="15.9" customHeight="1">
-      <c r="A46" s="72"/>
+      <c r="A46" s="70"/>
       <c r="B46" s="24" t="s">
         <v>14</v>
       </c>
@@ -2286,7 +2278,7 @@
       </c>
     </row>
     <row r="47" spans="1:6" ht="15.9" customHeight="1">
-      <c r="A47" s="72"/>
+      <c r="A47" s="70"/>
       <c r="B47" s="21" t="str">
         <f>$B$11</f>
         <v>Breeding of GM or HM</v>
@@ -2306,7 +2298,7 @@
       </c>
     </row>
     <row r="48" spans="1:6" ht="15.9" customHeight="1">
-      <c r="A48" s="73"/>
+      <c r="A48" s="71"/>
       <c r="B48" s="27" t="s">
         <v>6</v>
       </c>
@@ -2900,21 +2892,21 @@
       <c r="A82" s="16" t="s">
         <v>3</v>
       </c>
-      <c r="B82" s="86" t="s">
+      <c r="B82" s="84" t="s">
         <v>4</v>
       </c>
-      <c r="C82" s="81" t="s">
+      <c r="C82" s="79" t="s">
         <v>5</v>
       </c>
-      <c r="D82" s="82"/>
-      <c r="E82" s="83"/>
+      <c r="D82" s="80"/>
+      <c r="E82" s="81"/>
       <c r="F82" s="17" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="83" spans="1:6" ht="72.900000000000006" hidden="1" customHeight="1">
       <c r="A83" s="18"/>
-      <c r="B83" s="87"/>
+      <c r="B83" s="85"/>
       <c r="C83" s="19" t="s">
         <v>7</v>
       </c>
@@ -3407,7 +3399,7 @@
       </c>
     </row>
     <row r="108" spans="1:6" ht="15.9" customHeight="1">
-      <c r="A108" s="72" t="s">
+      <c r="A108" s="70" t="s">
         <v>34</v>
       </c>
       <c r="B108" s="21" t="s">
@@ -3428,7 +3420,7 @@
       </c>
     </row>
     <row r="109" spans="1:6" ht="15.9" customHeight="1">
-      <c r="A109" s="72"/>
+      <c r="A109" s="70"/>
       <c r="B109" s="24" t="s">
         <v>12</v>
       </c>
@@ -3447,7 +3439,7 @@
       </c>
     </row>
     <row r="110" spans="1:6" ht="15.9" customHeight="1">
-      <c r="A110" s="72"/>
+      <c r="A110" s="70"/>
       <c r="B110" s="21" t="s">
         <v>13</v>
       </c>
@@ -3466,7 +3458,7 @@
       </c>
     </row>
     <row r="111" spans="1:6" ht="15.9" customHeight="1">
-      <c r="A111" s="72"/>
+      <c r="A111" s="70"/>
       <c r="B111" s="24" t="s">
         <v>14</v>
       </c>
@@ -3485,7 +3477,7 @@
       </c>
     </row>
     <row r="112" spans="1:6" ht="15.9" customHeight="1">
-      <c r="A112" s="72"/>
+      <c r="A112" s="70"/>
       <c r="B112" s="21" t="str">
         <f>$B$11</f>
         <v>Breeding of GM or HM</v>
@@ -3505,7 +3497,7 @@
       </c>
     </row>
     <row r="113" spans="1:6" ht="15.9" customHeight="1">
-      <c r="A113" s="73"/>
+      <c r="A113" s="71"/>
       <c r="B113" s="27" t="s">
         <v>6</v>
       </c>
@@ -4401,21 +4393,21 @@
       <c r="A165" s="16" t="s">
         <v>3</v>
       </c>
-      <c r="B165" s="86" t="s">
+      <c r="B165" s="84" t="s">
         <v>4</v>
       </c>
-      <c r="C165" s="81" t="s">
+      <c r="C165" s="79" t="s">
         <v>5</v>
       </c>
-      <c r="D165" s="82"/>
-      <c r="E165" s="83"/>
+      <c r="D165" s="80"/>
+      <c r="E165" s="81"/>
       <c r="F165" s="17" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="166" spans="1:6" ht="72.900000000000006" hidden="1" customHeight="1">
       <c r="A166" s="18"/>
-      <c r="B166" s="87"/>
+      <c r="B166" s="85"/>
       <c r="C166" s="19" t="s">
         <v>7</v>
       </c>
@@ -4428,7 +4420,7 @@
       <c r="F166" s="20"/>
     </row>
     <row r="167" spans="1:6" ht="15.9" customHeight="1">
-      <c r="A167" s="72" t="s">
+      <c r="A167" s="70" t="s">
         <v>43</v>
       </c>
       <c r="B167" s="21" t="s">
@@ -4449,7 +4441,7 @@
       </c>
     </row>
     <row r="168" spans="1:6" ht="15.9" customHeight="1">
-      <c r="A168" s="72"/>
+      <c r="A168" s="70"/>
       <c r="B168" s="24" t="s">
         <v>12</v>
       </c>
@@ -4468,7 +4460,7 @@
       </c>
     </row>
     <row r="169" spans="1:6" ht="15.9" customHeight="1">
-      <c r="A169" s="72"/>
+      <c r="A169" s="70"/>
       <c r="B169" s="21" t="s">
         <v>13</v>
       </c>
@@ -4487,7 +4479,7 @@
       </c>
     </row>
     <row r="170" spans="1:6" ht="15.9" customHeight="1">
-      <c r="A170" s="72"/>
+      <c r="A170" s="70"/>
       <c r="B170" s="24" t="s">
         <v>14</v>
       </c>
@@ -4506,7 +4498,7 @@
       </c>
     </row>
     <row r="171" spans="1:6" ht="15.9" customHeight="1">
-      <c r="A171" s="72"/>
+      <c r="A171" s="70"/>
       <c r="B171" s="21" t="str">
         <f>$B$11</f>
         <v>Breeding of GM or HM</v>
@@ -4526,7 +4518,7 @@
       </c>
     </row>
     <row r="172" spans="1:6" ht="15.9" customHeight="1">
-      <c r="A172" s="73"/>
+      <c r="A172" s="71"/>
       <c r="B172" s="27" t="s">
         <v>6</v>
       </c>
@@ -4788,7 +4780,7 @@
       </c>
     </row>
     <row r="185" spans="1:6" ht="20.25" hidden="1" customHeight="1">
-      <c r="A185" s="74" t="s">
+      <c r="A185" s="72" t="s">
         <v>46</v>
       </c>
       <c r="B185" s="21" t="s">
@@ -4809,7 +4801,7 @@
       </c>
     </row>
     <row r="186" spans="1:6" ht="15.9" hidden="1" customHeight="1">
-      <c r="A186" s="75"/>
+      <c r="A186" s="73"/>
       <c r="B186" s="24" t="s">
         <v>12</v>
       </c>
@@ -5150,7 +5142,7 @@
       </c>
     </row>
     <row r="203" spans="1:6" ht="15.9" customHeight="1">
-      <c r="A203" s="72" t="s">
+      <c r="A203" s="70" t="s">
         <v>50</v>
       </c>
       <c r="B203" s="21" t="s">
@@ -5171,7 +5163,7 @@
       </c>
     </row>
     <row r="204" spans="1:6" ht="15.9" customHeight="1">
-      <c r="A204" s="72"/>
+      <c r="A204" s="70"/>
       <c r="B204" s="24" t="s">
         <v>12</v>
       </c>
@@ -5190,7 +5182,7 @@
       </c>
     </row>
     <row r="205" spans="1:6" ht="15.9" customHeight="1">
-      <c r="A205" s="72"/>
+      <c r="A205" s="70"/>
       <c r="B205" s="21" t="s">
         <v>13</v>
       </c>
@@ -5209,7 +5201,7 @@
       </c>
     </row>
     <row r="206" spans="1:6" ht="15.9" customHeight="1">
-      <c r="A206" s="72"/>
+      <c r="A206" s="70"/>
       <c r="B206" s="24" t="s">
         <v>14</v>
       </c>
@@ -5228,7 +5220,7 @@
       </c>
     </row>
     <row r="207" spans="1:6" ht="15.9" customHeight="1">
-      <c r="A207" s="72"/>
+      <c r="A207" s="70"/>
       <c r="B207" s="21" t="str">
         <f>$B$11</f>
         <v>Breeding of GM or HM</v>
@@ -5248,7 +5240,7 @@
       </c>
     </row>
     <row r="208" spans="1:6" ht="15.9" customHeight="1">
-      <c r="A208" s="73"/>
+      <c r="A208" s="71"/>
       <c r="B208" s="27" t="s">
         <v>6</v>
       </c>
@@ -5270,7 +5262,7 @@
       </c>
     </row>
     <row r="209" spans="1:6" ht="15.9" customHeight="1">
-      <c r="A209" s="72" t="s">
+      <c r="A209" s="70" t="s">
         <v>51</v>
       </c>
       <c r="B209" s="21" t="s">
@@ -5291,7 +5283,7 @@
       </c>
     </row>
     <row r="210" spans="1:6" ht="15.9" customHeight="1">
-      <c r="A210" s="72"/>
+      <c r="A210" s="70"/>
       <c r="B210" s="24" t="s">
         <v>12</v>
       </c>
@@ -5310,7 +5302,7 @@
       </c>
     </row>
     <row r="211" spans="1:6" ht="15.9" customHeight="1">
-      <c r="A211" s="72"/>
+      <c r="A211" s="70"/>
       <c r="B211" s="21" t="s">
         <v>13</v>
       </c>
@@ -5329,7 +5321,7 @@
       </c>
     </row>
     <row r="212" spans="1:6" ht="15.9" customHeight="1">
-      <c r="A212" s="72"/>
+      <c r="A212" s="70"/>
       <c r="B212" s="24" t="s">
         <v>14</v>
       </c>
@@ -5348,7 +5340,7 @@
       </c>
     </row>
     <row r="213" spans="1:6" ht="15.9" customHeight="1">
-      <c r="A213" s="72"/>
+      <c r="A213" s="70"/>
       <c r="B213" s="21" t="str">
         <f>$B$11</f>
         <v>Breeding of GM or HM</v>
@@ -5368,7 +5360,7 @@
       </c>
     </row>
     <row r="214" spans="1:6" ht="15.9" customHeight="1">
-      <c r="A214" s="73"/>
+      <c r="A214" s="71"/>
       <c r="B214" s="27" t="s">
         <v>6</v>
       </c>
@@ -5452,7 +5444,7 @@
       <c r="F220" s="23"/>
     </row>
     <row r="221" spans="1:6" ht="15.9" customHeight="1">
-      <c r="A221" s="76" t="s">
+      <c r="A221" s="74" t="s">
         <v>53</v>
       </c>
       <c r="B221" s="21" t="s">
@@ -5473,7 +5465,7 @@
       </c>
     </row>
     <row r="222" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A222" s="76"/>
+      <c r="A222" s="74"/>
       <c r="B222" s="24" t="s">
         <v>12</v>
       </c>
@@ -5492,7 +5484,7 @@
       </c>
     </row>
     <row r="223" spans="1:6" ht="15.9" customHeight="1">
-      <c r="A223" s="76"/>
+      <c r="A223" s="74"/>
       <c r="B223" s="21" t="s">
         <v>13</v>
       </c>
@@ -5511,7 +5503,7 @@
       </c>
     </row>
     <row r="224" spans="1:6" ht="18">
-      <c r="A224" s="76"/>
+      <c r="A224" s="74"/>
       <c r="B224" s="24" t="s">
         <v>14</v>
       </c>
@@ -5530,7 +5522,7 @@
       </c>
     </row>
     <row r="225" spans="1:6" ht="18">
-      <c r="A225" s="76"/>
+      <c r="A225" s="74"/>
       <c r="B225" s="21" t="str">
         <f>$B$11</f>
         <v>Breeding of GM or HM</v>
@@ -5550,7 +5542,7 @@
       </c>
     </row>
     <row r="226" spans="1:6" ht="18">
-      <c r="A226" s="77"/>
+      <c r="A226" s="75"/>
       <c r="B226" s="52" t="s">
         <v>54</v>
       </c>
@@ -5572,7 +5564,7 @@
       </c>
     </row>
     <row r="227" spans="1:6" ht="18" customHeight="1">
-      <c r="B227" s="70" t="s">
+      <c r="B227" s="66" t="s">
         <v>55</v>
       </c>
       <c r="C227" s="53">
@@ -5594,7 +5586,7 @@
     </row>
     <row r="228" spans="1:6" ht="18" customHeight="1">
       <c r="A228" s="54"/>
-      <c r="B228" s="70" t="s">
+      <c r="B228" s="66" t="s">
         <v>56</v>
       </c>
       <c r="C228" s="55">
@@ -5616,7 +5608,7 @@
     </row>
     <row r="229" spans="1:6" ht="18" customHeight="1">
       <c r="A229" s="57"/>
-      <c r="B229" s="70" t="s">
+      <c r="B229" s="66" t="s">
         <v>57</v>
       </c>
       <c r="C229" s="58">
@@ -5638,7 +5630,7 @@
     </row>
     <row r="230" spans="1:6" ht="18" customHeight="1">
       <c r="A230" s="57"/>
-      <c r="B230" s="71" t="s">
+      <c r="B230" s="67" t="s">
         <v>58</v>
       </c>
       <c r="C230" s="59">

</xml_diff>